<commit_message>
Update Vendor-Order-D652-18.04.2026 sample workbook
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/different sheets/Vendor-Order-D652-18.04.2026.xlsx
+++ b/different sheets/Vendor-Order-D652-18.04.2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://technocian-my.sharepoint.com/personal/sti_in_techno-design_net/Documents/Docs-2019/Sharad Personal/Auvera Studio/Buyer docs/PO-D652 - received-20-04-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiwar\Desktop\work\Shipping_software_Z\different sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80573BF3-9A39-4DD3-B919-7CB4F721CD00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A89376-B796-4BBF-8EF3-5C75A2B6E0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -19,19 +19,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Order!$A$1:$AK$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -168,6 +155,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>16</t>
     </r>
@@ -183,6 +171,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>18</t>
     </r>
@@ -199,6 +188,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>20</t>
     </r>
@@ -219,6 +209,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>22-24</t>
     </r>
@@ -239,6 +230,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>26-28</t>
     </r>
@@ -259,6 +251,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>30-32</t>
     </r>
@@ -279,6 +272,7 @@
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>34-36</t>
     </r>
@@ -412,46 +406,54 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
       <color rgb="FF00B0F0"/>
       <name val="Arial Rounded MT Bold"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -976,10 +978,16 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -988,31 +996,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1027,19 +1020,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1391,74 +1393,74 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AN22"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="5.85546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" style="1" customWidth="1"/>
-    <col min="9" max="24" width="6.42578125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.42578125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="7.7109375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="10.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6" max="7" width="5.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" style="1" customWidth="1"/>
+    <col min="9" max="24" width="6.44140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.44140625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="7.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="10.33203125" style="1" customWidth="1"/>
     <col min="28" max="28" width="13" style="1" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="8.140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="7.140625" style="1" customWidth="1"/>
-    <col min="32" max="33" width="11.5703125" style="1"/>
-    <col min="34" max="34" width="1.42578125" style="1" customWidth="1"/>
-    <col min="35" max="35" width="9.85546875" style="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" style="1"/>
-    <col min="37" max="37" width="8.28515625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="25.7109375" style="1" customWidth="1"/>
-    <col min="39" max="39" width="7.85546875" style="1" customWidth="1"/>
-    <col min="40" max="40" width="11.5703125" style="1"/>
+    <col min="29" max="29" width="10.33203125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="8.109375" style="1" customWidth="1"/>
+    <col min="31" max="31" width="7.109375" style="1" customWidth="1"/>
+    <col min="32" max="33" width="11.5546875" style="1"/>
+    <col min="34" max="34" width="1.44140625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="9.88671875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5546875" style="1"/>
+    <col min="37" max="37" width="8.33203125" style="1" customWidth="1"/>
+    <col min="38" max="38" width="25.6640625" style="1" customWidth="1"/>
+    <col min="39" max="39" width="7.88671875" style="1" customWidth="1"/>
+    <col min="40" max="40" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D1" s="69" t="s">
+    <row r="1" spans="1:40" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="Y1" s="68" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="Y1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
     </row>
-    <row r="2" spans="1:40" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:40" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="68"/>
+      <c r="Q2" s="68"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
@@ -1466,10 +1468,10 @@
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="4"/>
-      <c r="Y2" s="72" t="s">
+      <c r="Y2" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="Z2" s="73"/>
+      <c r="Z2" s="56"/>
       <c r="AA2" s="19"/>
       <c r="AB2" s="19"/>
       <c r="AC2" s="19"/>
@@ -1484,104 +1486,104 @@
       <c r="AL2" s="19"/>
       <c r="AM2" s="19"/>
     </row>
-    <row r="3" spans="1:40" ht="7.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="65" t="s">
+    <row r="3" spans="1:40" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="65" t="s">
+      <c r="B4" s="58"/>
+      <c r="C4" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="62"/>
       <c r="G4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="65" t="s">
+      <c r="H4" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="74"/>
-      <c r="J4" s="74"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="65" t="s">
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="74"/>
-      <c r="Q4" s="66"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="61"/>
+      <c r="O4" s="61"/>
+      <c r="P4" s="61"/>
+      <c r="Q4" s="58"/>
       <c r="R4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="S4" s="65" t="s">
+      <c r="S4" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="T4" s="74"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="66"/>
+      <c r="T4" s="61"/>
+      <c r="U4" s="61"/>
+      <c r="V4" s="61"/>
+      <c r="W4" s="61"/>
+      <c r="X4" s="61"/>
+      <c r="Y4" s="58"/>
       <c r="Z4" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="AA4" s="65" t="s">
+      <c r="AA4" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="AB4" s="66"/>
+      <c r="AB4" s="58"/>
     </row>
-    <row r="5" spans="1:40" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="57" t="str">
+    <row r="5" spans="1:40" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="59" t="str">
         <f>Y2</f>
         <v>D652</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="57" t="s">
+      <c r="B5" s="60"/>
+      <c r="C5" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="76"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="64"/>
       <c r="G5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="57" t="s">
+      <c r="H5" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="58"/>
-      <c r="L5" s="57" t="s">
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="60"/>
+      <c r="L5" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
-      <c r="Q5" s="58"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="63"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="63"/>
+      <c r="Q5" s="60"/>
       <c r="R5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="S5" s="57" t="s">
+      <c r="S5" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="T5" s="67"/>
-      <c r="U5" s="67"/>
-      <c r="V5" s="67"/>
-      <c r="W5" s="67"/>
-      <c r="X5" s="67"/>
-      <c r="Y5" s="58"/>
+      <c r="T5" s="63"/>
+      <c r="U5" s="63"/>
+      <c r="V5" s="63"/>
+      <c r="W5" s="63"/>
+      <c r="X5" s="63"/>
+      <c r="Y5" s="60"/>
       <c r="Z5" s="37"/>
-      <c r="AA5" s="57" t="s">
+      <c r="AA5" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="AB5" s="58"/>
+      <c r="AB5" s="60"/>
     </row>
-    <row r="6" spans="1:40" ht="7.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:40" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:40" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:40" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="53" t="s">
         <v>18</v>
       </c>
@@ -1636,7 +1638,7 @@
       <c r="AL7" s="28"/>
       <c r="AM7" s="31"/>
     </row>
-    <row r="8" spans="1:40" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:40" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="54"/>
       <c r="B8" s="16" t="s">
         <v>25</v>
@@ -1751,7 +1753,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:40" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:40" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>68</v>
       </c>
@@ -1834,7 +1836,7 @@
       <c r="AL9" s="30"/>
       <c r="AM9" s="24"/>
     </row>
-    <row r="10" spans="1:40" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:40" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>68</v>
       </c>
@@ -1917,8 +1919,8 @@
       <c r="AL10" s="30"/>
       <c r="AM10" s="24"/>
     </row>
-    <row r="11" spans="1:40" ht="3" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:40" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:40" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:40" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="33"/>
       <c r="B12" s="33"/>
       <c r="C12" s="34" t="s">
@@ -1963,7 +1965,7 @@
       <c r="AK12" s="34"/>
       <c r="AL12" s="34"/>
     </row>
-    <row r="13" spans="1:40" s="39" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:40" s="39" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="38"/>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -2005,53 +2007,53 @@
       <c r="AM13" s="38"/>
       <c r="AN13" s="38"/>
     </row>
-    <row r="14" spans="1:40" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="55" t="s">
+    <row r="14" spans="1:40" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="55" t="s">
+      <c r="B14" s="70"/>
+      <c r="C14" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="64"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="75"/>
+      <c r="F14" s="76"/>
       <c r="G14" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="55" t="s">
+      <c r="H14" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="63"/>
-      <c r="J14" s="63"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="55" t="s">
+      <c r="I14" s="75"/>
+      <c r="J14" s="75"/>
+      <c r="K14" s="70"/>
+      <c r="L14" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="M14" s="63"/>
-      <c r="N14" s="63"/>
-      <c r="O14" s="63"/>
-      <c r="P14" s="63"/>
-      <c r="Q14" s="56"/>
+      <c r="M14" s="75"/>
+      <c r="N14" s="75"/>
+      <c r="O14" s="75"/>
+      <c r="P14" s="75"/>
+      <c r="Q14" s="70"/>
       <c r="R14" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="S14" s="55" t="s">
+      <c r="S14" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="T14" s="63"/>
-      <c r="U14" s="63"/>
-      <c r="V14" s="63"/>
-      <c r="W14" s="63"/>
-      <c r="X14" s="63"/>
-      <c r="Y14" s="56"/>
+      <c r="T14" s="75"/>
+      <c r="U14" s="75"/>
+      <c r="V14" s="75"/>
+      <c r="W14" s="75"/>
+      <c r="X14" s="75"/>
+      <c r="Y14" s="70"/>
       <c r="Z14" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="AA14" s="55" t="s">
+      <c r="AA14" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="AB14" s="56"/>
+      <c r="AB14" s="70"/>
       <c r="AC14" s="38"/>
       <c r="AD14" s="38"/>
       <c r="AE14" s="38"/>
@@ -2065,51 +2067,51 @@
       <c r="AM14" s="38"/>
       <c r="AN14" s="38"/>
     </row>
-    <row r="15" spans="1:40" s="39" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="57" t="s">
+    <row r="15" spans="1:40" s="39" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="58"/>
-      <c r="C15" s="59" t="s">
+      <c r="B15" s="60"/>
+      <c r="C15" s="71" t="s">
         <v>79</v>
       </c>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="61"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="73"/>
       <c r="G15" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="59" t="s">
+      <c r="H15" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="62"/>
-      <c r="L15" s="59" t="s">
+      <c r="I15" s="72"/>
+      <c r="J15" s="72"/>
+      <c r="K15" s="74"/>
+      <c r="L15" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="M15" s="60"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60"/>
-      <c r="P15" s="60"/>
-      <c r="Q15" s="62"/>
+      <c r="M15" s="72"/>
+      <c r="N15" s="72"/>
+      <c r="O15" s="72"/>
+      <c r="P15" s="72"/>
+      <c r="Q15" s="74"/>
       <c r="R15" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="S15" s="59" t="s">
+      <c r="S15" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="T15" s="60"/>
-      <c r="U15" s="60"/>
-      <c r="V15" s="60"/>
-      <c r="W15" s="60"/>
-      <c r="X15" s="60"/>
-      <c r="Y15" s="62"/>
+      <c r="T15" s="72"/>
+      <c r="U15" s="72"/>
+      <c r="V15" s="72"/>
+      <c r="W15" s="72"/>
+      <c r="X15" s="72"/>
+      <c r="Y15" s="74"/>
       <c r="Z15" s="43"/>
-      <c r="AA15" s="59" t="s">
+      <c r="AA15" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="AB15" s="62"/>
+      <c r="AB15" s="74"/>
       <c r="AC15" s="38"/>
       <c r="AD15" s="38"/>
       <c r="AE15" s="38"/>
@@ -2123,7 +2125,7 @@
       <c r="AM15" s="38"/>
       <c r="AN15" s="38"/>
     </row>
-    <row r="16" spans="1:40" s="39" customFormat="1" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:40" s="39" customFormat="1" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="38"/>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
@@ -2165,7 +2167,7 @@
       <c r="AM16" s="38"/>
       <c r="AN16" s="38"/>
     </row>
-    <row r="17" spans="1:40" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:40" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="53" t="s">
         <v>18</v>
       </c>
@@ -2221,7 +2223,7 @@
       <c r="AM17" s="31"/>
       <c r="AN17" s="38"/>
     </row>
-    <row r="18" spans="1:40" s="39" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:40" s="39" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="54"/>
       <c r="B18" s="16" t="s">
         <v>25</v>
@@ -2337,7 +2339,7 @@
       </c>
       <c r="AN18" s="38"/>
     </row>
-    <row r="19" spans="1:40" s="39" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:40" s="39" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>68</v>
       </c>
@@ -2421,7 +2423,7 @@
       <c r="AM19" s="48"/>
       <c r="AN19" s="38"/>
     </row>
-    <row r="20" spans="1:40" s="39" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:40" s="39" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="38"/>
       <c r="B20" s="38"/>
       <c r="C20" s="38"/>
@@ -2463,7 +2465,7 @@
       <c r="AM20" s="38"/>
       <c r="AN20" s="38"/>
     </row>
-    <row r="21" spans="1:40" s="39" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:40" s="39" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="49"/>
       <c r="B21" s="49"/>
       <c r="C21" s="50" t="s">
@@ -2510,7 +2512,7 @@
       <c r="AM21" s="38"/>
       <c r="AN21" s="38"/>
     </row>
-    <row r="22" spans="1:40" s="39" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:40" s="39" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="38"/>
       <c r="B22" s="38"/>
       <c r="C22" s="52"/>
@@ -2555,22 +2557,6 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="29">
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="Y2:Z2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="H4:K4"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="L4:Q4"/>
-    <mergeCell ref="L5:Q5"/>
-    <mergeCell ref="S4:Y4"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="S5:Y5"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="D1:Q2"/>
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="AA14:AB14"/>
     <mergeCell ref="A15:B15"/>
@@ -2584,6 +2570,22 @@
     <mergeCell ref="H14:K14"/>
     <mergeCell ref="L14:Q14"/>
     <mergeCell ref="S14:Y14"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="S5:Y5"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="D1:Q2"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="Y2:Z2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="L4:Q4"/>
+    <mergeCell ref="L5:Q5"/>
+    <mergeCell ref="S4:Y4"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="58" fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>